<commit_message>
feat: promotion-wide diploma ranking and S3 XLSX export
</commit_message>
<xml_diff>
--- a/src/main/resources/xlsx/diplomas_all.xlsx
+++ b/src/main/resources/xlsx/diplomas_all.xlsx
@@ -104,27 +104,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>STD21006</t>
+          <t>STD21001</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Razafy</t>
+          <t>Rakoto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Nirina</t>
+          <t>Hery</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>13.00</t>
+          <t>14.00</t>
         </is>
       </c>
     </row>
@@ -136,17 +136,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>STD21001</t>
+          <t>STD21003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Rakoto</t>
+          <t>Andria</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Hery</t>
+          <t>Tiana</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -158,34 +158,34 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>STD21003</t>
+          <t>STD21006</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Andria</t>
+          <t>Razafy</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tiana</t>
+          <t>Nirina</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>14.00</t>
+          <t>13.00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">

</xml_diff>